<commit_message>
📝 Update GSP1146 sample with completely fresh, original mock data instead of lab copy
</commit_message>
<xml_diff>
--- a/tutorials/Episode-09-GSP1146/GSP1146.xlsx
+++ b/tutorials/Episode-09-GSP1146/GSP1146.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,134 +473,134 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0d5ff8cd8d</t>
+          <t>8af694cfd9</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Fredrick</t>
+          <t>Aarav</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thompson</t>
+          <t>Kumar</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>33562</t>
+          <t>26238</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>fredrick.thompson@fakeitcompany.com</t>
+          <t>aarav.kumar@mockcustomer.com</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ATM wont turn on</t>
+          <t>ATM screen frozen</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ATM screen is black</t>
+          <t>Customer reported atm screen frozen at branch.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Hardware Failure</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Shelley Gomez</t>
+          <t>Rahul Sharma</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>d9c1547599</t>
+          <t>c881367b93</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Patsy</t>
+          <t>Sophia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sheehan</t>
+          <t>Davis</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>66722</t>
+          <t>85775</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>patsy.sheehan@fakeitcompany.com</t>
+          <t>sophia.davis@mockcustomer.com</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Card reader not working</t>
+          <t>Cash dispenser not dispensing</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>The ATM is not recognizing cards</t>
+          <t>Customer reported cash dispenser not dispensing at branch.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Dispenser Issues</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Justin Sato</t>
+          <t>Amit Patel</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e0cb653f42</t>
+          <t>2980e332f2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jon</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Snow</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3351</t>
+          <t>20409</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>jon.snow@fakeitcompany.com</t>
+          <t>michael.smith@mockcustomer.com</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Broken keypad</t>
+          <t>Keypad unresponsive</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>The 2 on the keypad isn't working</t>
+          <t>Customer reported keypad unresponsive at branch.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -610,189 +610,189 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Shelley Gomez</t>
+          <t>Sarah Connor</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>94803beda8</t>
+          <t>7663dc177a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alexander</t>
+          <t>Aarav</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ramos</t>
+          <t>Kumar</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>37490</t>
+          <t>44069</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>alexander.ramos@fakeitcompany.com</t>
+          <t>aarav.kumar@mockcustomer.com</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Low cash supply</t>
+          <t>Network timeout</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ATM dispensed 2 $10 bills, instead of 1 $20 bill</t>
+          <t>Customer reported network timeout at branch.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Cash Dispenser</t>
+          <t>Connectivity</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Miles Barnes</t>
+          <t>Amit Patel</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>da18217bc3</t>
+          <t>22b1664e0b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verna</t>
+          <t>Emma</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Moore</t>
+          <t>Johnson</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>77827</t>
+          <t>57430</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>verna.moore@fakeitcompany.com</t>
+          <t>emma.johnson@mockcustomer.com</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Cash dispenser jam</t>
+          <t>ATM screen frozen</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Cash is stuck</t>
+          <t>Customer reported atm screen frozen at branch.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Cash Dispenser</t>
+          <t>Hardware Failure</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Miles Barnes</t>
+          <t>Priya Singh</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>d146f1ccc1</t>
+          <t>a9c7bcc315</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Megan</t>
+          <t>Neha</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Iverson</t>
+          <t>Gupta</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>51428</t>
+          <t>94912</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>megan.iverson@fakeitcompany.com</t>
+          <t>neha.gupta@mockcustomer.com</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Connection error</t>
+          <t>Receipt printer jammed</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Cannot connect to bank's network</t>
+          <t>Customer reported receipt printer jammed at branch.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Connection error</t>
+          <t>Printing</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Nia Jones</t>
+          <t>John Doe</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>045dbe3b7b</t>
+          <t>0fea5da2cc</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Sophia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Edson</t>
+          <t>Davis</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>16252</t>
+          <t>29253</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>paul.edson@fakeitcompany.com</t>
+          <t>sophia.davis@mockcustomer.com</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Keypad unresponsive</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>ATM is not recognizing a correct PIN</t>
+          <t>Customer reported keypad unresponsive at branch.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -802,183 +802,295 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Justin Sato</t>
+          <t>Amit Patel</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>d9d1df320a</t>
+          <t>d96506125a</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Danielle</t>
+          <t>Emma</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>Johnson</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>98308</t>
+          <t>48394</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>danielle.west@fakeitcompany.com</t>
+          <t>emma.johnson@mockcustomer.com</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Receipt printer out of paper</t>
+          <t>Cash dispenser not dispensing</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Receipt didn't print</t>
+          <t>Customer reported cash dispenser not dispensing at branch.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Receipts</t>
+          <t>Dispenser Issues</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Jean Clark</t>
+          <t>Priya Singh</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JTXhApOb</t>
+          <t>18cc0654b1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alexander</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ramos</t>
+          <t>Miller</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>37490</t>
+          <t>30081</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>alexander.ramos@fakeitcompany.com</t>
+          <t>lucas.miller@mockcustomer.com</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Receipt printer out of ink</t>
+          <t>Card reader swallowed card</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Receipt printed blank</t>
+          <t>Customer reported card reader swallowed card at branch.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Receipts</t>
+          <t>Hardware Failure</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Jean Clark</t>
+          <t>Rahul Sharma</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>23a5558b</t>
+          <t>de1cfc768a</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>quick</t>
+          <t>Aarav</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>lab</t>
+          <t>Kumar</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ABC123</t>
+          <t>17420</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>student-01-41527e028127@qwiklabs.net</t>
+          <t>aarav.kumar@mockcustomer.com</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Card reader not working</t>
+          <t>Network timeout</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Customer reported network timeout at branch.</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Connectivity</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Shelley Gomez</t>
+          <t>Rahul Sharma</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ac7aa33f</t>
+          <t>cd88e58b96</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Freeda</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>Oliver</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Freeda123</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>34774</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>oliver.brown@mockcustomer.com</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Receipt printer out of ink</t>
+          <t>Receipt paper out</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Customer reported receipt paper out at branch.</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Receipts</t>
+          <t>Printing</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Jean Clark</t>
+          <t>Sarah Connor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>b747829946</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kavya</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Joshi</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>92731</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>kavya.joshi@mockcustomer.com</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Keypad unresponsive</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Customer reported keypad unresponsive at branch.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>General Issues</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Amit Patel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1c6fc5de96</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>quick</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>lab</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ABC123</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>student-01-mock@qwiklabs.net</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Receipt paper out</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Lab testing ticket</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Printing</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Priya Singh</t>
         </is>
       </c>
     </row>
@@ -1021,17 +1133,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Shelley Gomez</t>
+          <t>Rahul Sharma</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>shelley.gomez@fakeitcompany.com</t>
+          <t>rahul.sharma@examplebank.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>555-0101</t>
+          <t>9876543210</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1043,17 +1155,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Justin Sato</t>
+          <t>Priya Singh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>justin.sato@fakeitcompany.com</t>
+          <t>priya.singh@examplebank.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>555-0102</t>
+          <t>9876543211</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1065,17 +1177,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Miles Barnes</t>
+          <t>Amit Patel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>miles.barnes@fakeitcompany.com</t>
+          <t>amit.patel@examplebank.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>555-0103</t>
+          <t>9876543212</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1087,17 +1199,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Nia Jones</t>
+          <t>Sarah Connor</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>nia.jones@fakeitcompany.com</t>
+          <t>sarah.connor@examplebank.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>555-0104</t>
+          <t>9876543213</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1109,17 +1221,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jean Clark</t>
+          <t>John Doe</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>jean.clark@fakeitcompany.com</t>
+          <t>john.doe@examplebank.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>555-0105</t>
+          <t>9876543214</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1157,108 +1269,108 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ATM wont turn on</t>
+          <t>ATM screen frozen</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Hardware Failure</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Card reader not working</t>
+          <t>Card reader swallowed card</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Hardware Failure</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Broken keypad</t>
+          <t>Cash dispenser not dispensing</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Dispenser Issues</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Low cash supply</t>
+          <t>Dispensed incorrect amount</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cash Dispenser</t>
+          <t>Dispenser Issues</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cash dispenser jam</t>
+          <t>Network timeout</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cash Dispenser</t>
+          <t>Connectivity</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Connection error</t>
+          <t>Cannot connect to server</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Connection error</t>
+          <t>Connectivity</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Receipt printer jammed</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Printing</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Receipt printer out of paper</t>
+          <t>Receipt paper out</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Receipts</t>
+          <t>Printing</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Receipt printer out of ink</t>
+          <t>Keypad unresponsive</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Receipts</t>
+          <t>General Issues</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📝 Revert GSP1146 sample data to exactly match the Qwiklabs backend requirements
</commit_message>
<xml_diff>
--- a/tutorials/Episode-09-GSP1146/GSP1146.xlsx
+++ b/tutorials/Episode-09-GSP1146/GSP1146.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,134 +473,134 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8af694cfd9</t>
+          <t>0d5ff8cd8d</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aarav</t>
+          <t>Fredrick</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Kumar</t>
+          <t>Thompson</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>26238</t>
+          <t>33562</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>aarav.kumar@mockcustomer.com</t>
+          <t>fredrick.thompson@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ATM screen frozen</t>
+          <t>ATM wont turn on</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Customer reported atm screen frozen at branch.</t>
+          <t>ATM screen is black</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Hardware Failure</t>
+          <t>General Issues</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Rahul Sharma</t>
+          <t>Shelley Gomez</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>c881367b93</t>
+          <t>d9c1547599</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sophia</t>
+          <t>Patsy</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Sheehan</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>85775</t>
+          <t>66722</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>sophia.davis@mockcustomer.com</t>
+          <t>patsy.sheehan@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cash dispenser not dispensing</t>
+          <t>Card reader not working</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Customer reported cash dispenser not dispensing at branch.</t>
+          <t>The ATM is not recognizing cards</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Dispenser Issues</t>
+          <t>General Issues</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Amit Patel</t>
+          <t>Justin Sato</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2980e332f2</t>
+          <t>e0cb653f42</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Jon</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Snow</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>20409</t>
+          <t>3351</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>michael.smith@mockcustomer.com</t>
+          <t>jon.snow@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Keypad unresponsive</t>
+          <t>Broken keypad</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Customer reported keypad unresponsive at branch.</t>
+          <t>The 2 on the keypad isn't working</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -610,189 +610,189 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Sarah Connor</t>
+          <t>Shelley Gomez</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7663dc177a</t>
+          <t>94803beda8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aarav</t>
+          <t>Alexander</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kumar</t>
+          <t>Ramos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>44069</t>
+          <t>37490</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>aarav.kumar@mockcustomer.com</t>
+          <t>alexander.ramos@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Network timeout</t>
+          <t>Low cash supply</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Customer reported network timeout at branch.</t>
+          <t>ATM dispensed 2 $10 bills, instead of 1 $20 bill</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Connectivity</t>
+          <t>Cash Dispenser</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Amit Patel</t>
+          <t>Miles Barnes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>22b1664e0b</t>
+          <t>da18217bc3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Emma</t>
+          <t>Verna</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Moore</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>57430</t>
+          <t>77827</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>emma.johnson@mockcustomer.com</t>
+          <t>verna.moore@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ATM screen frozen</t>
+          <t>Cash dispenser jam</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Customer reported atm screen frozen at branch.</t>
+          <t>Cash is stuck</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Hardware Failure</t>
+          <t>Cash Dispenser</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Priya Singh</t>
+          <t>Miles Barnes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>a9c7bcc315</t>
+          <t>d146f1ccc1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Neha</t>
+          <t>Megan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gupta</t>
+          <t>Iverson</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>94912</t>
+          <t>51428</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>neha.gupta@mockcustomer.com</t>
+          <t>megan.iverson@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Receipt printer jammed</t>
+          <t>Connection error</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Customer reported receipt printer jammed at branch.</t>
+          <t>Cannot connect to bank's network</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Printing</t>
+          <t>Connection error</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Nia Jones</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0fea5da2cc</t>
+          <t>045dbe3b7b</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sophia</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Edson</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>29253</t>
+          <t>16252</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>sophia.davis@mockcustomer.com</t>
+          <t>paul.edson@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Keypad unresponsive</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Customer reported keypad unresponsive at branch.</t>
+          <t>ATM is not recognizing a correct PIN</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -802,295 +802,183 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Amit Patel</t>
+          <t>Justin Sato</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>d96506125a</t>
+          <t>d9d1df320a</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Emma</t>
+          <t>Danielle</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>West</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>48394</t>
+          <t>98308</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>emma.johnson@mockcustomer.com</t>
+          <t>danielle.west@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Cash dispenser not dispensing</t>
+          <t>Receipt printer out of paper</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Customer reported cash dispenser not dispensing at branch.</t>
+          <t>Receipt didn't print</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Dispenser Issues</t>
+          <t>Receipts</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Priya Singh</t>
+          <t>Jean Clark</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18cc0654b1</t>
+          <t>JTXhApOb</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Alexander</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Miller</t>
+          <t>Ramos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>30081</t>
+          <t>37490</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>lucas.miller@mockcustomer.com</t>
+          <t>alexander.ramos@fakeitcompany.com</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Card reader swallowed card</t>
+          <t>Receipt printer out of ink</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Customer reported card reader swallowed card at branch.</t>
+          <t>Receipt printed blank</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Hardware Failure</t>
+          <t>Receipts</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Rahul Sharma</t>
+          <t>Jean Clark</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>de1cfc768a</t>
+          <t>23a5558b</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Aarav</t>
+          <t>quick</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kumar</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>17420</t>
+          <t>ABC123</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>aarav.kumar@mockcustomer.com</t>
+          <t>student-01-41527e028127@qwiklabs.net</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Network timeout</t>
+          <t>Card reader not working</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Customer reported network timeout at branch.</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Connectivity</t>
+          <t>General Issues</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Rahul Sharma</t>
+          <t>Shelley Gomez</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cd88e58b96</t>
+          <t>ac7aa33f</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Oliver</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Brown</t>
-        </is>
-      </c>
+          <t>Freeda</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>34774</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>oliver.brown@mockcustomer.com</t>
-        </is>
-      </c>
+          <t>Freeda123</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Receipt paper out</t>
+          <t>Receipt printer out of ink</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Customer reported receipt paper out at branch.</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Printing</t>
+          <t>Receipts</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Sarah Connor</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>b747829946</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Kavya</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Joshi</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>92731</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>kavya.joshi@mockcustomer.com</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Keypad unresponsive</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Customer reported keypad unresponsive at branch.</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>General Issues</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Amit Patel</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1c6fc5de96</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>quick</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>lab</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>ABC123</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>student-01-mock@qwiklabs.net</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Receipt paper out</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Lab testing ticket</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Printing</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Priya Singh</t>
+          <t>Jean Clark</t>
         </is>
       </c>
     </row>
@@ -1133,17 +1021,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rahul Sharma</t>
+          <t>Shelley Gomez</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>rahul.sharma@examplebank.com</t>
+          <t>shelley.gomez@fakeitcompany.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>555-0101</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1155,17 +1043,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Priya Singh</t>
+          <t>Justin Sato</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>priya.singh@examplebank.com</t>
+          <t>justin.sato@fakeitcompany.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9876543211</t>
+          <t>555-0102</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1177,17 +1065,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Amit Patel</t>
+          <t>Miles Barnes</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>amit.patel@examplebank.com</t>
+          <t>miles.barnes@fakeitcompany.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9876543212</t>
+          <t>555-0103</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1199,17 +1087,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sarah Connor</t>
+          <t>Nia Jones</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sarah.connor@examplebank.com</t>
+          <t>nia.jones@fakeitcompany.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>9876543213</t>
+          <t>555-0104</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1221,17 +1109,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Jean Clark</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>john.doe@examplebank.com</t>
+          <t>jean.clark@fakeitcompany.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>9876543214</t>
+          <t>555-0105</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1269,108 +1157,108 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ATM screen frozen</t>
+          <t>ATM wont turn on</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hardware Failure</t>
+          <t>General Issues</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Card reader swallowed card</t>
+          <t>Card reader not working</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hardware Failure</t>
+          <t>General Issues</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cash dispenser not dispensing</t>
+          <t>Broken keypad</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dispenser Issues</t>
+          <t>General Issues</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dispensed incorrect amount</t>
+          <t>Low cash supply</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dispenser Issues</t>
+          <t>Cash Dispenser</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Network timeout</t>
+          <t>Cash dispenser jam</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Connectivity</t>
+          <t>Cash Dispenser</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cannot connect to server</t>
+          <t>Connection error</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Connectivity</t>
+          <t>Connection error</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Receipt printer jammed</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Printing</t>
+          <t>General Issues</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Receipt paper out</t>
+          <t>Receipt printer out of paper</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Printing</t>
+          <t>Receipts</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Keypad unresponsive</t>
+          <t>Receipt printer out of ink</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>General Issues</t>
+          <t>Receipts</t>
         </is>
       </c>
     </row>

</xml_diff>